<commit_message>
emp details from excel
</commit_message>
<xml_diff>
--- a/tests/testdata/HRM.xlsx
+++ b/tests/testdata/HRM.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GCS\My_GCS_AUTOMATION\tests\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GCS\seleniumLearn1\tests\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3362BD8C-ED4E-481A-8807-5AFCFF4CB4B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7CCFBD-F80F-4609-8887-BE5CE63B8D26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{19F5FA6D-8631-47F2-9D2E-C372D3A7140D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{19F5FA6D-8631-47F2-9D2E-C372D3A7140D}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="emp" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>password</t>
   </si>
@@ -48,19 +49,43 @@
   </si>
   <si>
     <t>userid</t>
+  </si>
+  <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>middlename</t>
+  </si>
+  <si>
+    <t>lastname</t>
+  </si>
+  <si>
+    <t>FName1</t>
+  </si>
+  <si>
+    <t>MName1</t>
+  </si>
+  <si>
+    <t>LName1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF6AAB73"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -83,8 +108,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -420,9 +448,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D2C8DEB-9F82-4143-AD07-0456BD420654}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -430,12 +458,44 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F37AEAB4-02B5-47F5-AF73-A72185D7112F}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>